<commit_message>
Aggiunta comunicazione seriale 10bit. Funziona con commit "ec32ff2".
</commit_message>
<xml_diff>
--- a/db/ike_params_process_data.xlsx
+++ b/db/ike_params_process_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr codeName="Questa_cartella_di_lavoro" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucag\local_repos\ike_gui\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F14B140-5716-4A37-B6AB-FE785A8E0F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{145C36BA-318D-425C-9A48-9C61151E7076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{35ECC9C5-EA02-4EE7-AAE2-09095EF705F3}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{35ECC9C5-EA02-4EE7-AAE2-09095EF705F3}"/>
   </bookViews>
   <sheets>
     <sheet name="params_data" sheetId="9" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="fixed_point" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">process_data!$A$1:$N$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">process_data!$A$1:$N$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -248,9 +248,6 @@
     <t>word allarme 1</t>
   </si>
   <si>
-    <t>diagn_out.scr_synch_invalid_cnt</t>
-  </si>
-  <si>
     <t>tensione uscita (rms)</t>
   </si>
   <si>
@@ -467,7 +464,10 @@
     <t>contatore isr freq_in_update</t>
   </si>
   <si>
-    <t>01.02.05</t>
+    <t>scr_out.scr_synch_invalid_cnt</t>
+  </si>
+  <si>
+    <t>01.02.06</t>
   </si>
 </sst>
 </file>
@@ -915,7 +915,7 @@
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>17</v>
@@ -942,16 +942,16 @@
         <v>1</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O1" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
@@ -1043,10 +1043,10 @@
         <v>23</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M3" s="7">
         <f t="shared" si="0"/>
@@ -1102,7 +1102,7 @@
         <v>24</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M4" s="7">
         <f t="shared" si="0"/>
@@ -1130,7 +1130,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="D5" s="1">
         <v>3</v>
@@ -1155,10 +1155,10 @@
         <v>30</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="M5" s="7">
         <f>65535/(I5-H5)</f>
@@ -1214,7 +1214,7 @@
         <v>31</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="M6" s="7">
         <f>65535/(I6-H6)</f>
@@ -1270,7 +1270,7 @@
         <v>32</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M7" s="7">
         <f>65535/(I7-H7)</f>
@@ -1320,13 +1320,13 @@
         <v>65535</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>33</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M8" s="7">
         <f>65535/(I8-H8)</f>
@@ -1376,13 +1376,13 @@
         <v>65535</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>34</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M9" s="7">
         <f t="shared" si="0"/>
@@ -1435,10 +1435,10 @@
         <v>23</v>
       </c>
       <c r="K10" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="L10" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>124</v>
       </c>
       <c r="M10" s="7">
         <f t="shared" ref="M10" si="6">65535/(I10-H10)</f>
@@ -1494,7 +1494,7 @@
         <v>35</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="M11" s="7">
         <f t="shared" si="0"/>
@@ -1550,7 +1550,7 @@
         <v>36</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M12" s="7">
         <f t="shared" si="0"/>
@@ -1606,7 +1606,7 @@
         <v>37</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="M13" s="7">
         <f t="shared" si="0"/>
@@ -1656,13 +1656,13 @@
         <v>65535</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K14" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="L14" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>126</v>
       </c>
       <c r="M14" s="7">
         <f t="shared" ref="M14" si="10">65535/(I14-H14)</f>
@@ -1712,7 +1712,7 @@
         <v>1</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>38</v>
@@ -1824,7 +1824,7 @@
         <v>1</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>40</v>
@@ -1995,10 +1995,10 @@
         <v>23</v>
       </c>
       <c r="K20" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="L20" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>136</v>
       </c>
       <c r="M20" s="7">
         <f t="shared" ref="M20" si="15">65535/(I20-H20)</f>
@@ -2054,7 +2054,7 @@
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>16</v>
@@ -2075,16 +2075,16 @@
         <v>1</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M1" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="N1" s="11" t="s">
         <v>75</v>
-      </c>
-      <c r="N1" s="11" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
@@ -2120,7 +2120,7 @@
         <v>58</v>
       </c>
       <c r="K2" s="7">
-        <f t="shared" ref="K2:K26" si="0">65535/(G2-F2)</f>
+        <f t="shared" ref="K2:K25" si="0">65535/(G2-F2)</f>
         <v>1</v>
       </c>
       <c r="L2" s="7">
@@ -2128,7 +2128,7 @@
         <v>1</v>
       </c>
       <c r="M2" s="7">
-        <f t="shared" ref="M2:M26" si="1">1/K2</f>
+        <f t="shared" ref="M2:M25" si="1">1/K2</f>
         <v>1</v>
       </c>
       <c r="N2" s="14">
@@ -2173,7 +2173,7 @@
         <v>1</v>
       </c>
       <c r="L3" s="7">
-        <f t="shared" ref="L3:L26" si="2">1/K3</f>
+        <f t="shared" ref="L3:L25" si="2">1/K3</f>
         <v>1</v>
       </c>
       <c r="M3" s="7">
@@ -2181,7 +2181,7 @@
         <v>1</v>
       </c>
       <c r="N3" s="14">
-        <f t="shared" ref="N3:N26" si="3">ROUND((E3-F3)*K3,0)</f>
+        <f t="shared" ref="N3:N25" si="3">ROUND((E3-F3)*K3,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2212,10 +2212,10 @@
         <v>27</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K4" s="7">
         <f t="shared" si="0"/>
@@ -2261,10 +2261,10 @@
         <v>28</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K5" s="7">
         <f t="shared" si="0"/>
@@ -2310,10 +2310,10 @@
         <v>27</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K6" s="7">
         <f t="shared" si="0"/>
@@ -2359,10 +2359,10 @@
         <v>28</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="K7" s="7">
         <f t="shared" si="0"/>
@@ -2411,7 +2411,7 @@
         <v>63</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K8" s="7">
         <f t="shared" si="0"/>
@@ -2460,7 +2460,7 @@
         <v>64</v>
       </c>
       <c r="J9" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K9" s="7">
         <f t="shared" si="0"/>
@@ -2503,13 +2503,13 @@
         <v>100</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I10" s="11" t="s">
         <v>62</v>
       </c>
       <c r="J10" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K10" s="7">
         <f t="shared" si="0"/>
@@ -2555,10 +2555,10 @@
         <v>26</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J11" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" si="0"/>
@@ -2601,13 +2601,13 @@
         <v>65535</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I12" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="J12" s="11" t="s">
         <v>127</v>
-      </c>
-      <c r="J12" s="11" t="s">
-        <v>128</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" ref="K12" si="5">65535/(G12-F12)</f>
@@ -2650,13 +2650,13 @@
         <v>65535</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" ref="K13" si="9">65535/(G13-F13)</f>
@@ -2699,13 +2699,13 @@
         <v>65535</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" ref="K14" si="13">65535/(G14-F14)</f>
@@ -2748,13 +2748,13 @@
         <v>65535</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>23</v>
+        <v>76</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="0"/>
@@ -2895,13 +2895,13 @@
         <v>65535</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I18" s="11" t="s">
         <v>85</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="0"/>
@@ -2944,13 +2944,13 @@
         <v>65535</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="0"/>
@@ -2993,13 +2993,13 @@
         <v>65535</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="0"/>
@@ -3090,11 +3090,11 @@
       <c r="G22" s="1">
         <v>65535</v>
       </c>
-      <c r="H22" s="12" t="s">
-        <v>81</v>
+      <c r="H22" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="J22" s="11" t="s">
         <v>105</v>
@@ -3143,25 +3143,25 @@
         <v>23</v>
       </c>
       <c r="I23" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="J23" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="J23" s="11" t="s">
-        <v>106</v>
-      </c>
       <c r="K23" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="K23" si="17">65535/(G23-F23)</f>
         <v>1</v>
       </c>
       <c r="L23" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="L23" si="18">1/K23</f>
         <v>1</v>
       </c>
       <c r="M23" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="M23" si="19">1/K23</f>
         <v>1</v>
       </c>
       <c r="N23" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="N23" si="20">ROUND((E23-F23)*K23,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3171,46 +3171,46 @@
         <v>41</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="D24" s="1">
-        <v>0</v>
-      </c>
-      <c r="E24" s="1">
-        <v>0</v>
-      </c>
-      <c r="F24" s="1">
-        <v>0</v>
-      </c>
-      <c r="G24" s="1">
-        <v>65535</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>23</v>
+        <v>2</v>
+      </c>
+      <c r="E24" s="3">
+        <v>0</v>
+      </c>
+      <c r="F24" s="3">
+        <v>0</v>
+      </c>
+      <c r="G24" s="3">
+        <v>1</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>25</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>107</v>
+        <v>60</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="K24" s="7">
-        <f t="shared" ref="K24" si="17">65535/(G24-F24)</f>
-        <v>1</v>
+        <f>65535/(G24-F24)</f>
+        <v>65535</v>
       </c>
       <c r="L24" s="7">
-        <f t="shared" ref="L24" si="18">1/K24</f>
-        <v>1</v>
+        <f>1/K24</f>
+        <v>1.5259021896696422E-5</v>
       </c>
       <c r="M24" s="7">
-        <f t="shared" ref="M24" si="19">1/K24</f>
-        <v>1</v>
+        <f>1/K24</f>
+        <v>1.5259021896696422E-5</v>
       </c>
       <c r="N24" s="14">
-        <f t="shared" ref="N24" si="20">ROUND((E24-F24)*K24,0)</f>
+        <f>ROUND((E24-F24)*K24,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3226,7 +3226,7 @@
         <v>50</v>
       </c>
       <c r="D25" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E25" s="3">
         <v>0</v>
@@ -3235,31 +3235,31 @@
         <v>0</v>
       </c>
       <c r="G25" s="3">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="K25" s="7">
-        <f>65535/(G25-F25)</f>
-        <v>65535</v>
+        <f t="shared" si="0"/>
+        <v>1008.2307692307693</v>
       </c>
       <c r="L25" s="7">
-        <f>1/K25</f>
-        <v>1.5259021896696422E-5</v>
+        <f t="shared" si="2"/>
+        <v>9.9183642328526736E-4</v>
       </c>
       <c r="M25" s="7">
-        <f>1/K25</f>
-        <v>1.5259021896696422E-5</v>
+        <f t="shared" si="1"/>
+        <v>9.9183642328526736E-4</v>
       </c>
       <c r="N25" s="14">
-        <f>ROUND((E25-F25)*K25,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3272,48 +3272,48 @@
         <v>53</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="D26" s="1">
-        <v>3</v>
-      </c>
-      <c r="E26" s="3">
-        <v>0</v>
-      </c>
-      <c r="F26" s="3">
-        <v>0</v>
-      </c>
-      <c r="G26" s="3">
-        <v>65</v>
-      </c>
-      <c r="H26" s="11" t="s">
-        <v>26</v>
+        <v>0</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0</v>
+      </c>
+      <c r="F26" s="1">
+        <v>0</v>
+      </c>
+      <c r="G26" s="1">
+        <v>65535</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>23</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
       <c r="K26" s="7">
-        <f t="shared" si="0"/>
-        <v>1008.2307692307693</v>
+        <f t="shared" ref="K26" si="21">65535/(G26-F26)</f>
+        <v>1</v>
       </c>
       <c r="L26" s="7">
-        <f t="shared" si="2"/>
-        <v>9.9183642328526736E-4</v>
+        <f t="shared" ref="L26" si="22">1/K26</f>
+        <v>1</v>
       </c>
       <c r="M26" s="7">
-        <f t="shared" si="1"/>
-        <v>9.9183642328526736E-4</v>
+        <f t="shared" ref="M26" si="23">1/K26</f>
+        <v>1</v>
       </c>
       <c r="N26" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="N26" si="24">ROUND((E26-F26)*K26,0)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N26" xr:uid="{931DECF4-8BF0-4C1D-87E4-E5713582A1AF}"/>
+  <autoFilter ref="A1:N25" xr:uid="{931DECF4-8BF0-4C1D-87E4-E5713582A1AF}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>